<commit_message>
adicion de casos de prueba
</commit_message>
<xml_diff>
--- a/Gestíon/3.1.3 Planilla Casos de Prueba.xlsx
+++ b/Gestíon/3.1.3 Planilla Casos de Prueba.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luism\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\VAMOS-\Gestíon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70FFDC28-ED4E-43E5-8D10-5D3FF4504776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F50996CE-D004-4C75-B053-22ACE8B1B161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -161,7 +161,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="249">
   <si>
     <t>Casos de Pruebas Estándar</t>
   </si>
@@ -671,6 +671,291 @@
   </si>
   <si>
     <t>La aplicación consume la Directions API de Google Maps y dibuja una ruta exacta desde la ubicación del usuario hasta las coordenadas del evento.</t>
+  </si>
+  <si>
+    <t>Unirse a grupo con código de invitación</t>
+  </si>
+  <si>
+    <t>Validar el flujo del Usuario B uniéndose a un grupo existente mediante el invite_code generado por el Usuario A en CP-04.</t>
+  </si>
+  <si>
+    <t>1. Usuario A comparte el invite_code (generado en CP-04) con Usuario B vía WhatsApp.</t>
+  </si>
+  <si>
+    <t>invite_code válido generado previamente.</t>
+  </si>
+  <si>
+    <t>El código llega íntegro al Usuario B.</t>
+  </si>
+  <si>
+    <t>2. Usuario B (sesión activa) entra a "Mis Eventos" y presiona "Unirse a grupo".</t>
+  </si>
+  <si>
+    <t>Se despliega el JoinGroupModal con el input de código.</t>
+  </si>
+  <si>
+    <t>3. Usuario B ingresa el invite_code y confirma.</t>
+  </si>
+  <si>
+    <t>invite_code copiado del Usuario A.</t>
+  </si>
+  <si>
+    <t>Backend valida, agrega al Usuario B al grupo, confirma automáticamente el evento en su lista y refresca la vista.</t>
+  </si>
+  <si>
+    <t>Validación de edad límite (exactamente 18 años)</t>
+  </si>
+  <si>
+    <t>Verificar el comportamiento exacto del límite inferior de la regla de edad (&gt;= 18) como caso borde.</t>
+  </si>
+  <si>
+    <t>1. Iniciar sesión con Google con una cuenta nueva.</t>
+  </si>
+  <si>
+    <t>Cuenta Google nueva válida.</t>
+  </si>
+  <si>
+    <t>2. Ingresar una fecha que resulte en exactamente 18 años cumplidos hoy (fecha actual menos 18 años exactos) y confirmar.</t>
+  </si>
+  <si>
+    <t>Fecha de nacimiento = 21/06/2008</t>
+  </si>
+  <si>
+    <t>El sistema acepta el registro porque la regla es &gt;= 18 (no &gt; 18). Usuario redirigido al mapa.</t>
+  </si>
+  <si>
+    <t>Persistencia de sesión JWT entre aperturas</t>
+  </si>
+  <si>
+    <t>Comprobar que el JWT almacenado en expo-secure-store mantenga la sesión activa al reabrir la app.</t>
+  </si>
+  <si>
+    <t>1. Iniciar sesión con un usuario válido y verificar acceso al mapa.</t>
+  </si>
+  <si>
+    <t>Cuenta válida.</t>
+  </si>
+  <si>
+    <t>Acceso correcto a la pantalla principal.</t>
+  </si>
+  <si>
+    <t>2. Cerrar la aplicación por completo (deslizar fuera del multitasking).</t>
+  </si>
+  <si>
+    <t>La app se cierra correctamente.</t>
+  </si>
+  <si>
+    <t>3. Volver a abrir la app.</t>
+  </si>
+  <si>
+    <t>La app recupera el JWT desde expo-secure-store, valida el token y redirige directamente al mapa sin solicitar nuevo login.</t>
+  </si>
+  <si>
+    <t>Distinción entre Guardar y Confirmar eventos</t>
+  </si>
+  <si>
+    <t>Eventos / Listas personales</t>
+  </si>
+  <si>
+    <t>Verificar que las acciones "Guardar" y "Confirmar" del EventDetailSheet gestionen listas independientes.</t>
+  </si>
+  <si>
+    <t>1. Tocar un marcador del mapa para abrir el EventDetailSheet.</t>
+  </si>
+  <si>
+    <t>Mapa con eventos visibles.</t>
+  </si>
+  <si>
+    <t>Se despliega la ficha del evento con ambos botones disponibles.</t>
+  </si>
+  <si>
+    <t>2. Presionar "Guardar" en el primer evento.</t>
+  </si>
+  <si>
+    <t>El marcador cambia a estado "guardado" y el SavedEventsContext registra el evento.</t>
+  </si>
+  <si>
+    <t>3. Tocar otro marcador y presionar "Confirmar".</t>
+  </si>
+  <si>
+    <t>Mapa con al menos 2 eventos.</t>
+  </si>
+  <si>
+    <t>El marcador cambia a estado "confirmado".</t>
+  </si>
+  <si>
+    <t>4. Ir a la pestaña "Mis Eventos".</t>
+  </si>
+  <si>
+    <t>Cada evento aparece en su lista correspondiente (Guardados / Confirmados) sin mezclarse.</t>
+  </si>
+  <si>
+    <t>Filtro de eventos por rango de fecha (DateSelector)</t>
+  </si>
+  <si>
+    <t>Validar el filtrado dinámico de marcadores según el rango "Hoy / Semana / Mes" del DateSelector.</t>
+  </si>
+  <si>
+    <t>1. Abrir la pestaña "Mapa" con el filtro en "Mes" (default).</t>
+  </si>
+  <si>
+    <t>BD con eventos en distintas fechas del mes.</t>
+  </si>
+  <si>
+    <t>Se renderizan todos los eventos del mes en curso.</t>
+  </si>
+  <si>
+    <t>2. Cambiar el filtro a "Semana".</t>
+  </si>
+  <si>
+    <t>El mapa vuelve a renderizar mostrando solo eventos dentro de los próximos 7 días.</t>
+  </si>
+  <si>
+    <t>3. Cambiar el filtro a "Hoy".</t>
+  </si>
+  <si>
+    <t>El mapa renderiza únicamente los eventos cuya fecha_evento coincide con el día actual.</t>
+  </si>
+  <si>
+    <t>Cambio de modo de transporte en la ruta</t>
+  </si>
+  <si>
+    <t>Verificar el cambio de modo de viaje (caminando / auto / transporte) en el RoutePanel y la actualización del cálculo.</t>
+  </si>
+  <si>
+    <t>1. Activar "Cómo llegar" desde un evento.</t>
+  </si>
+  <si>
+    <t>GPS activo, evento alcanzable.</t>
+  </si>
+  <si>
+    <t>Se dibuja la ruta inicial y se despliega el RoutePanel.</t>
+  </si>
+  <si>
+    <t>2. Cambiar el modo a "Caminando".</t>
+  </si>
+  <si>
+    <t>Google Directions recalcula. Se actualiza distancia (km), tiempo estimado e instrucciones paso a paso.</t>
+  </si>
+  <si>
+    <t>3. Cambiar el modo a "Auto".</t>
+  </si>
+  <si>
+    <t>Google Directions recalcula con el nuevo modo. Datos del panel actualizados.</t>
+  </si>
+  <si>
+    <t>4. Cambiar el modo a "Transporte".</t>
+  </si>
+  <si>
+    <t>Se calcula ruta con transporte público (en español). Panel refleja los nuevos tiempos.</t>
+  </si>
+  <si>
+    <t>Estados de miembros del grupo (EstadoModal)</t>
+  </si>
+  <si>
+    <t>Confirmar que cada uno de los 5 estados posibles se persista correctamente y se refleje visualmente.</t>
+  </si>
+  <si>
+    <t>1. Abrir el EstadoModal del grupo.</t>
+  </si>
+  <si>
+    <t>Usuario activo en un grupo logístico.</t>
+  </si>
+  <si>
+    <t>Se despliegan las 5 opciones: Aún no salgo / En camino / Llegué / Esperando fuera / Cancelé.</t>
+  </si>
+  <si>
+    <t>2. Seleccionar "Aún no salgo" y confirmar.</t>
+  </si>
+  <si>
+    <t>PATCH al backend, estado persistido en PostgreSQL, ícono visual del usuario actualizado.</t>
+  </si>
+  <si>
+    <t>3. Repetir el cambio para "En camino", "Llegué", "Esperando fuera" y "Cancelé".</t>
+  </si>
+  <si>
+    <t>Cada cambio refleja el ícono correcto y persiste correctamente sin errores intermedios.</t>
+  </si>
+  <si>
+    <t>Vambot con prompt vacío (manejo de errores)</t>
+  </si>
+  <si>
+    <t>No Funcional - Robustez</t>
+  </si>
+  <si>
+    <t>Validar que la app maneje correctamente un prompt vacío o solo con espacios, sin enviar la consulta a Gemini.</t>
+  </si>
+  <si>
+    <t>Sesión activa, Vambot disponible.</t>
+  </si>
+  <si>
+    <t>Se despliega la interfaz de chat.</t>
+  </si>
+  <si>
+    <t>2. Sin escribir nada (o solo espacios en blanco), intentar presionar el botón de enviar.</t>
+  </si>
+  <si>
+    <t>El frontend bloquea el envío (botón deshabilitado o validación local). No se gastan tokens de Gemini ni se muestra error en la UI.</t>
+  </si>
+  <si>
+    <t>Manejo de permisos de ubicación denegados</t>
+  </si>
+  <si>
+    <t>Mapa / Ubicación</t>
+  </si>
+  <si>
+    <t>Verificar el comportamiento de la app cuando el usuario deniega los permisos de GPS.</t>
+  </si>
+  <si>
+    <t>1. Desde la configuración del SO, denegar los permisos de ubicación a VAMOS!.</t>
+  </si>
+  <si>
+    <t>Permisos de ubicación = Denegados.</t>
+  </si>
+  <si>
+    <t>Permisos correctamente revocados en el SO.</t>
+  </si>
+  <si>
+    <t>2. Abrir la app e iniciar sesión.</t>
+  </si>
+  <si>
+    <t>Sesión válida.</t>
+  </si>
+  <si>
+    <t>La app carga sin crashear. El mapa se centra en una ubicación por defecto (Providencia).</t>
+  </si>
+  <si>
+    <t>3. Tocar un evento e intentar usar la funcionalidad "Cómo llegar".</t>
+  </si>
+  <si>
+    <t>La app muestra un mensaje controlado indicando que se requieren permisos de ubicación. No hay crash ni pantalla en blanco.</t>
+  </si>
+  <si>
+    <t>El usuario fue agregado al grupo exitosamente mediante el código, confirmando el evento en su lista personal y actualizando la interfaz. (Pass).</t>
+  </si>
+  <si>
+    <t>El sistema aceptó el registro correctamente al validar la condición de límite inferior (&gt;= 18) y redirigió al mapa principal. (Pass).</t>
+  </si>
+  <si>
+    <t>El token fue recuperado exitosamente desde expo-secure-store, restaurando la sesión activa de forma automática sin requerir un nuevo login. (Pass).</t>
+  </si>
+  <si>
+    <t>Los eventos fueron asignados a sus listas correspondientes (Guardados / Confirmados) de forma completamente independiente y sin cruce de datos. (Pass).</t>
+  </si>
+  <si>
+    <t>El mapa actualizó y renderizó dinámicamente los marcadores reflejando con exactitud los eventos correspondientes al rango de tiempo seleccionado. (Pass).</t>
+  </si>
+  <si>
+    <t>La ruta fue recalculada exitosamente por la API según el nuevo modo de viaje, actualizando con precisión la distancia, el tiempo y las instrucciones. (Pass).</t>
+  </si>
+  <si>
+    <t>Cada actualización de estado fue persistida correctamente en la base de datos y reflejada visualmente en el ícono del usuario sin interrupciones. (Pass).</t>
+  </si>
+  <si>
+    <t>El frontend bloqueó exitosamente el envío de la petición vacía, previniendo el consumo innecesario de la API y manteniendo la estabilidad de la UI. (Pass).</t>
+  </si>
+  <si>
+    <t>La aplicación manejó la falta de permisos correctamente sin crashear, mostrando el mensaje de advertencia controlado al intentar calcular la ruta. (Pass).</t>
   </si>
 </sst>
 </file>
@@ -1361,7 +1646,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1493,55 +1778,132 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="26" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="22" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="26" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="22" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="28" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1564,6 +1926,9 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="26" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1573,85 +1938,8 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="26" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="22" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="26" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="22" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2351,6 +2639,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>323850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="AutoShape 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21460999-0005-BAA9-1390-8E154E2168AD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7620000" cy="8362950"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2701,10 +3043,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1">
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="63"/>
+      <c r="C1" s="83"/>
       <c r="D1" s="44"/>
       <c r="E1" s="44"/>
       <c r="F1" s="44"/>
@@ -2730,11 +3072,11 @@
       <c r="J2" s="41"/>
     </row>
     <row r="3" spans="1:15" ht="18" customHeight="1">
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="68"/>
-      <c r="D3" s="69"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="74"/>
       <c r="E3" s="37"/>
       <c r="F3" s="37"/>
       <c r="G3" s="37"/>
@@ -2743,11 +3085,11 @@
       <c r="J3" s="37"/>
     </row>
     <row r="4" spans="1:15" ht="17.25" thickBot="1">
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="71"/>
       <c r="E4" s="38"/>
       <c r="F4" s="37"/>
       <c r="G4" s="37"/>
@@ -2770,10 +3112,10 @@
       <c r="A6" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="59" t="s">
+      <c r="B6" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="60"/>
+      <c r="C6" s="80"/>
       <c r="D6" s="51" t="s">
         <v>5</v>
       </c>
@@ -2788,11 +3130,11 @@
       <c r="A7" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="62"/>
-      <c r="D7" s="83" t="s">
+      <c r="C7" s="76"/>
+      <c r="D7" s="55" t="s">
         <v>75</v>
       </c>
       <c r="E7" s="33"/>
@@ -2801,11 +3143,11 @@
       <c r="A8" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="55" t="s">
+      <c r="B8" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="56"/>
-      <c r="D8" s="84" t="s">
+      <c r="C8" s="78"/>
+      <c r="D8" s="56" t="s">
         <v>75</v>
       </c>
       <c r="E8" s="33"/>
@@ -2814,103 +3156,103 @@
       <c r="A9" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="56"/>
-      <c r="D9" s="84" t="s">
+      <c r="C9" s="78"/>
+      <c r="D9" s="56" t="s">
         <v>75</v>
       </c>
       <c r="E9" s="33"/>
     </row>
     <row r="10" spans="1:15" ht="15" customHeight="1">
       <c r="A10" s="28"/>
-      <c r="B10" s="55"/>
-      <c r="C10" s="56"/>
+      <c r="B10" s="77"/>
+      <c r="C10" s="78"/>
       <c r="D10" s="32"/>
       <c r="E10" s="33"/>
     </row>
     <row r="11" spans="1:15" ht="15" customHeight="1">
       <c r="A11" s="28"/>
-      <c r="B11" s="55"/>
-      <c r="C11" s="56"/>
+      <c r="B11" s="77"/>
+      <c r="C11" s="78"/>
       <c r="D11" s="32"/>
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:15" ht="15" customHeight="1">
       <c r="A12" s="28"/>
-      <c r="B12" s="55"/>
-      <c r="C12" s="56"/>
+      <c r="B12" s="77"/>
+      <c r="C12" s="78"/>
       <c r="D12" s="32"/>
       <c r="E12" s="33"/>
     </row>
     <row r="13" spans="1:15" ht="15" customHeight="1">
       <c r="A13" s="28"/>
-      <c r="B13" s="55"/>
-      <c r="C13" s="56"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="78"/>
       <c r="D13" s="32"/>
       <c r="E13" s="33"/>
     </row>
     <row r="14" spans="1:15" ht="15" customHeight="1">
       <c r="A14" s="28"/>
-      <c r="B14" s="55"/>
-      <c r="C14" s="56"/>
+      <c r="B14" s="77"/>
+      <c r="C14" s="78"/>
       <c r="D14" s="32"/>
       <c r="E14" s="33"/>
     </row>
     <row r="15" spans="1:15" ht="15" customHeight="1">
       <c r="A15" s="28"/>
-      <c r="B15" s="55"/>
-      <c r="C15" s="56"/>
+      <c r="B15" s="77"/>
+      <c r="C15" s="78"/>
       <c r="D15" s="32"/>
       <c r="E15" s="33"/>
     </row>
     <row r="16" spans="1:15" ht="15" customHeight="1">
       <c r="A16" s="28"/>
-      <c r="B16" s="55"/>
-      <c r="C16" s="56"/>
+      <c r="B16" s="77"/>
+      <c r="C16" s="78"/>
       <c r="D16" s="32"/>
       <c r="E16" s="33"/>
     </row>
     <row r="17" spans="1:5" ht="15" customHeight="1">
       <c r="A17" s="28"/>
-      <c r="B17" s="55"/>
-      <c r="C17" s="56"/>
+      <c r="B17" s="77"/>
+      <c r="C17" s="78"/>
       <c r="D17" s="32"/>
       <c r="E17" s="33"/>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1">
       <c r="A18" s="28"/>
-      <c r="B18" s="55"/>
-      <c r="C18" s="56"/>
+      <c r="B18" s="77"/>
+      <c r="C18" s="78"/>
       <c r="D18" s="32"/>
       <c r="E18" s="33"/>
     </row>
     <row r="19" spans="1:5" ht="15" customHeight="1">
       <c r="A19" s="28"/>
-      <c r="B19" s="55"/>
-      <c r="C19" s="56"/>
+      <c r="B19" s="77"/>
+      <c r="C19" s="78"/>
       <c r="D19" s="32"/>
       <c r="E19" s="33"/>
     </row>
     <row r="20" spans="1:5" ht="15" customHeight="1">
       <c r="A20" s="28"/>
-      <c r="B20" s="55"/>
-      <c r="C20" s="56"/>
+      <c r="B20" s="77"/>
+      <c r="C20" s="78"/>
       <c r="D20" s="32"/>
       <c r="E20" s="33"/>
     </row>
     <row r="21" spans="1:5" ht="15" customHeight="1">
       <c r="A21" s="28"/>
-      <c r="B21" s="55"/>
-      <c r="C21" s="56"/>
+      <c r="B21" s="77"/>
+      <c r="C21" s="78"/>
       <c r="D21" s="32"/>
       <c r="E21" s="33"/>
     </row>
     <row r="22" spans="1:5" ht="15" customHeight="1" thickBot="1">
       <c r="A22" s="26"/>
-      <c r="B22" s="57"/>
-      <c r="C22" s="58"/>
+      <c r="B22" s="81"/>
+      <c r="C22" s="82"/>
       <c r="D22" s="31"/>
       <c r="E22" s="33"/>
     </row>
@@ -2922,10 +3264,10 @@
       <c r="A24" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="59" t="s">
+      <c r="B24" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="60"/>
+      <c r="C24" s="80"/>
       <c r="D24" s="52"/>
       <c r="E24" s="33"/>
     </row>
@@ -2933,11 +3275,11 @@
       <c r="A25" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="61" t="s">
+      <c r="B25" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="62"/>
-      <c r="D25" s="85" t="s">
+      <c r="C25" s="76"/>
+      <c r="D25" s="57" t="s">
         <v>75</v>
       </c>
       <c r="E25" s="33"/>
@@ -2946,11 +3288,11 @@
       <c r="A26" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="55" t="s">
+      <c r="B26" s="77" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="56"/>
-      <c r="D26" s="84" t="s">
+      <c r="C26" s="78"/>
+      <c r="D26" s="56" t="s">
         <v>75</v>
       </c>
       <c r="E26" s="33"/>
@@ -2959,98 +3301,98 @@
       <c r="A27" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="55" t="s">
+      <c r="B27" s="77" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="56"/>
-      <c r="D27" s="84" t="s">
+      <c r="C27" s="78"/>
+      <c r="D27" s="56" t="s">
         <v>76</v>
       </c>
       <c r="E27" s="33"/>
     </row>
     <row r="28" spans="1:5" ht="15" customHeight="1">
       <c r="A28" s="28"/>
-      <c r="B28" s="55"/>
-      <c r="C28" s="56"/>
+      <c r="B28" s="77"/>
+      <c r="C28" s="78"/>
       <c r="D28" s="32"/>
       <c r="E28" s="33"/>
     </row>
     <row r="29" spans="1:5" ht="15" customHeight="1">
       <c r="A29" s="28"/>
-      <c r="B29" s="55"/>
-      <c r="C29" s="56"/>
+      <c r="B29" s="77"/>
+      <c r="C29" s="78"/>
       <c r="D29" s="32"/>
     </row>
     <row r="30" spans="1:5" ht="15" customHeight="1">
       <c r="A30" s="28"/>
-      <c r="B30" s="55"/>
-      <c r="C30" s="56"/>
+      <c r="B30" s="77"/>
+      <c r="C30" s="78"/>
       <c r="D30" s="32"/>
     </row>
     <row r="31" spans="1:5" ht="15" customHeight="1">
       <c r="A31" s="28"/>
-      <c r="B31" s="55"/>
-      <c r="C31" s="56"/>
+      <c r="B31" s="77"/>
+      <c r="C31" s="78"/>
       <c r="D31" s="32"/>
     </row>
     <row r="32" spans="1:5" ht="15" customHeight="1">
       <c r="A32" s="28"/>
-      <c r="B32" s="55"/>
-      <c r="C32" s="56"/>
+      <c r="B32" s="77"/>
+      <c r="C32" s="78"/>
       <c r="D32" s="32"/>
     </row>
     <row r="33" spans="1:4" ht="15" customHeight="1">
       <c r="A33" s="28"/>
-      <c r="B33" s="55"/>
-      <c r="C33" s="56"/>
+      <c r="B33" s="77"/>
+      <c r="C33" s="78"/>
       <c r="D33" s="32"/>
     </row>
     <row r="34" spans="1:4" ht="15" customHeight="1">
       <c r="A34" s="28"/>
-      <c r="B34" s="55"/>
-      <c r="C34" s="56"/>
+      <c r="B34" s="77"/>
+      <c r="C34" s="78"/>
       <c r="D34" s="32"/>
     </row>
     <row r="35" spans="1:4" ht="15" customHeight="1">
       <c r="A35" s="28"/>
-      <c r="B35" s="55"/>
-      <c r="C35" s="56"/>
+      <c r="B35" s="77"/>
+      <c r="C35" s="78"/>
       <c r="D35" s="32"/>
     </row>
     <row r="36" spans="1:4" ht="15" customHeight="1">
       <c r="A36" s="28"/>
-      <c r="B36" s="55"/>
-      <c r="C36" s="56"/>
+      <c r="B36" s="77"/>
+      <c r="C36" s="78"/>
       <c r="D36" s="32"/>
     </row>
     <row r="37" spans="1:4" ht="15" customHeight="1">
       <c r="A37" s="28"/>
-      <c r="B37" s="55"/>
-      <c r="C37" s="56"/>
+      <c r="B37" s="77"/>
+      <c r="C37" s="78"/>
       <c r="D37" s="32"/>
     </row>
     <row r="38" spans="1:4" ht="15" customHeight="1">
       <c r="A38" s="28"/>
-      <c r="B38" s="55"/>
-      <c r="C38" s="56"/>
+      <c r="B38" s="77"/>
+      <c r="C38" s="78"/>
       <c r="D38" s="32"/>
     </row>
     <row r="39" spans="1:4" ht="15" customHeight="1">
       <c r="A39" s="28"/>
-      <c r="B39" s="55"/>
-      <c r="C39" s="56"/>
+      <c r="B39" s="77"/>
+      <c r="C39" s="78"/>
       <c r="D39" s="32"/>
     </row>
     <row r="40" spans="1:4" ht="15" customHeight="1">
       <c r="A40" s="28"/>
-      <c r="B40" s="55"/>
-      <c r="C40" s="56"/>
+      <c r="B40" s="77"/>
+      <c r="C40" s="78"/>
       <c r="D40" s="32"/>
     </row>
     <row r="41" spans="1:4" ht="15" customHeight="1" thickBot="1">
       <c r="A41" s="26"/>
-      <c r="B41" s="57"/>
-      <c r="C41" s="58"/>
+      <c r="B41" s="81"/>
+      <c r="C41" s="82"/>
       <c r="D41" s="31"/>
     </row>
     <row r="42" spans="1:4" ht="20.100000000000001" customHeight="1" thickBot="1"/>
@@ -3058,21 +3400,21 @@
       <c r="A43" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B43" s="59" t="s">
+      <c r="B43" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C43" s="60"/>
+      <c r="C43" s="80"/>
       <c r="D43" s="53"/>
     </row>
     <row r="44" spans="1:4" ht="15" customHeight="1">
       <c r="A44" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="B44" s="61" t="s">
+      <c r="B44" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="62"/>
-      <c r="D44" s="85" t="s">
+      <c r="C44" s="76"/>
+      <c r="D44" s="57" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3080,11 +3422,11 @@
       <c r="A45" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B45" s="55" t="s">
+      <c r="B45" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="C45" s="56"/>
-      <c r="D45" s="84" t="s">
+      <c r="C45" s="78"/>
+      <c r="D45" s="56" t="s">
         <v>75</v>
       </c>
     </row>
@@ -3092,84 +3434,84 @@
       <c r="A46" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="B46" s="55" t="s">
+      <c r="B46" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="C46" s="56"/>
-      <c r="D46" s="84" t="s">
+      <c r="C46" s="78"/>
+      <c r="D46" s="56" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15" customHeight="1">
       <c r="A47" s="28"/>
-      <c r="B47" s="55"/>
-      <c r="C47" s="56"/>
+      <c r="B47" s="77"/>
+      <c r="C47" s="78"/>
       <c r="D47" s="28"/>
     </row>
     <row r="48" spans="1:4" ht="15" customHeight="1">
       <c r="A48" s="28"/>
-      <c r="B48" s="55"/>
-      <c r="C48" s="56"/>
+      <c r="B48" s="77"/>
+      <c r="C48" s="78"/>
       <c r="D48" s="28"/>
     </row>
     <row r="49" spans="1:4" ht="15" customHeight="1">
       <c r="A49" s="28"/>
-      <c r="B49" s="55"/>
-      <c r="C49" s="56"/>
+      <c r="B49" s="77"/>
+      <c r="C49" s="78"/>
       <c r="D49" s="28"/>
     </row>
     <row r="50" spans="1:4" ht="15" customHeight="1">
       <c r="A50" s="28"/>
-      <c r="B50" s="55"/>
-      <c r="C50" s="56"/>
+      <c r="B50" s="77"/>
+      <c r="C50" s="78"/>
       <c r="D50" s="28"/>
     </row>
     <row r="51" spans="1:4" ht="15" customHeight="1">
       <c r="A51" s="28"/>
-      <c r="B51" s="55"/>
-      <c r="C51" s="56"/>
+      <c r="B51" s="77"/>
+      <c r="C51" s="78"/>
       <c r="D51" s="28"/>
     </row>
     <row r="52" spans="1:4" ht="15" customHeight="1">
       <c r="A52" s="28"/>
-      <c r="B52" s="55"/>
-      <c r="C52" s="56"/>
+      <c r="B52" s="77"/>
+      <c r="C52" s="78"/>
       <c r="D52" s="28"/>
     </row>
     <row r="53" spans="1:4" ht="15" customHeight="1">
       <c r="A53" s="28"/>
-      <c r="B53" s="55"/>
-      <c r="C53" s="56"/>
+      <c r="B53" s="77"/>
+      <c r="C53" s="78"/>
       <c r="D53" s="28"/>
     </row>
     <row r="54" spans="1:4" ht="15" customHeight="1">
       <c r="A54" s="28"/>
-      <c r="B54" s="55"/>
-      <c r="C54" s="56"/>
+      <c r="B54" s="77"/>
+      <c r="C54" s="78"/>
       <c r="D54" s="28"/>
     </row>
     <row r="55" spans="1:4" ht="15" customHeight="1">
       <c r="A55" s="28"/>
-      <c r="B55" s="55"/>
-      <c r="C55" s="56"/>
+      <c r="B55" s="77"/>
+      <c r="C55" s="78"/>
       <c r="D55" s="28"/>
     </row>
     <row r="56" spans="1:4" ht="15" customHeight="1">
       <c r="A56" s="28"/>
-      <c r="B56" s="55"/>
-      <c r="C56" s="56"/>
+      <c r="B56" s="77"/>
+      <c r="C56" s="78"/>
       <c r="D56" s="28"/>
     </row>
     <row r="57" spans="1:4" ht="15" customHeight="1">
       <c r="A57" s="28"/>
-      <c r="B57" s="55"/>
-      <c r="C57" s="56"/>
+      <c r="B57" s="77"/>
+      <c r="C57" s="78"/>
       <c r="D57" s="28"/>
     </row>
     <row r="58" spans="1:4" ht="15" customHeight="1" thickBot="1">
       <c r="A58" s="26"/>
-      <c r="B58" s="57"/>
-      <c r="C58" s="58"/>
+      <c r="B58" s="81"/>
+      <c r="C58" s="82"/>
       <c r="D58" s="26"/>
     </row>
     <row r="59" spans="1:4" ht="20.100000000000001" customHeight="1" thickBot="1"/>
@@ -3177,21 +3519,21 @@
       <c r="A60" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B60" s="59" t="s">
+      <c r="B60" s="79" t="s">
         <v>26</v>
       </c>
-      <c r="C60" s="60"/>
+      <c r="C60" s="80"/>
       <c r="D60" s="53"/>
     </row>
     <row r="61" spans="1:4" ht="15" customHeight="1">
       <c r="A61" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="B61" s="61" t="s">
+      <c r="B61" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="C61" s="62"/>
-      <c r="D61" s="84" t="s">
+      <c r="C61" s="76"/>
+      <c r="D61" s="56" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3199,11 +3541,11 @@
       <c r="A62" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="B62" s="55" t="s">
+      <c r="B62" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="C62" s="56"/>
-      <c r="D62" s="84" t="s">
+      <c r="C62" s="78"/>
+      <c r="D62" s="56" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3215,7 +3557,7 @@
         <v>32</v>
       </c>
       <c r="C63" s="49"/>
-      <c r="D63" s="84" t="s">
+      <c r="D63" s="56" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3239,8 +3581,8 @@
     </row>
     <row r="67" spans="1:4" ht="15" customHeight="1" thickBot="1">
       <c r="A67" s="26"/>
-      <c r="B67" s="57"/>
-      <c r="C67" s="58"/>
+      <c r="B67" s="81"/>
+      <c r="C67" s="82"/>
       <c r="D67" s="26"/>
     </row>
     <row r="68" spans="1:4" ht="15" customHeight="1">
@@ -3251,21 +3593,21 @@
       <c r="A70" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B70" s="59" t="s">
+      <c r="B70" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="C70" s="60"/>
+      <c r="C70" s="80"/>
       <c r="D70" s="53"/>
     </row>
     <row r="71" spans="1:4" ht="15" customHeight="1">
       <c r="A71" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="B71" s="61" t="s">
+      <c r="B71" s="75" t="s">
         <v>35</v>
       </c>
-      <c r="C71" s="62"/>
-      <c r="D71" s="83" t="s">
+      <c r="C71" s="76"/>
+      <c r="D71" s="55" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3273,11 +3615,11 @@
       <c r="A72" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="B72" s="55" t="s">
+      <c r="B72" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="C72" s="56"/>
-      <c r="D72" s="84" t="s">
+      <c r="C72" s="78"/>
+      <c r="D72" s="56" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3295,20 +3637,20 @@
     </row>
     <row r="75" spans="1:4" ht="15" customHeight="1">
       <c r="A75" s="28"/>
-      <c r="B75" s="55"/>
-      <c r="C75" s="56"/>
+      <c r="B75" s="77"/>
+      <c r="C75" s="78"/>
       <c r="D75" s="28"/>
     </row>
     <row r="76" spans="1:4" ht="15" customHeight="1">
       <c r="A76" s="28"/>
-      <c r="B76" s="55"/>
-      <c r="C76" s="56"/>
+      <c r="B76" s="77"/>
+      <c r="C76" s="78"/>
       <c r="D76" s="28"/>
     </row>
     <row r="77" spans="1:4" ht="15" customHeight="1" thickBot="1">
       <c r="A77" s="26"/>
-      <c r="B77" s="57"/>
-      <c r="C77" s="58"/>
+      <c r="B77" s="81"/>
+      <c r="C77" s="82"/>
       <c r="D77" s="26"/>
     </row>
     <row r="78" spans="1:4" ht="20.100000000000001" customHeight="1" thickBot="1"/>
@@ -3316,40 +3658,40 @@
       <c r="A79" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B79" s="59" t="s">
+      <c r="B79" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="C79" s="60"/>
+      <c r="C79" s="80"/>
       <c r="D79" s="53"/>
     </row>
     <row r="80" spans="1:4" ht="14.25">
-      <c r="A80" s="86" t="s">
+      <c r="A80" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="B80" s="87" t="s">
+      <c r="B80" s="84" t="s">
         <v>77</v>
       </c>
-      <c r="C80" s="87"/>
+      <c r="C80" s="84"/>
       <c r="D80" s="29"/>
     </row>
     <row r="81" spans="1:4" ht="14.25">
-      <c r="A81" s="88" t="s">
+      <c r="A81" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="B81" s="89" t="s">
+      <c r="B81" s="85" t="s">
         <v>78</v>
       </c>
-      <c r="C81" s="89"/>
+      <c r="C81" s="85"/>
       <c r="D81" s="29"/>
     </row>
     <row r="82" spans="1:4" ht="14.25">
-      <c r="A82" s="88" t="s">
+      <c r="A82" s="59" t="s">
         <v>41</v>
       </c>
-      <c r="B82" s="90" t="s">
+      <c r="B82" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="C82" s="91"/>
+      <c r="C82" s="61"/>
       <c r="D82" s="29"/>
     </row>
     <row r="83" spans="1:4" ht="14.25">
@@ -3365,20 +3707,20 @@
       <c r="D84" s="29"/>
     </row>
     <row r="85" spans="1:4" ht="14.25">
-      <c r="B85" s="55"/>
-      <c r="C85" s="56"/>
+      <c r="B85" s="77"/>
+      <c r="C85" s="78"/>
       <c r="D85" s="28"/>
     </row>
     <row r="86" spans="1:4" ht="14.25">
       <c r="A86" s="28"/>
-      <c r="B86" s="55"/>
-      <c r="C86" s="56"/>
+      <c r="B86" s="77"/>
+      <c r="C86" s="78"/>
       <c r="D86" s="27"/>
     </row>
     <row r="87" spans="1:4" ht="15" thickBot="1">
       <c r="A87" s="26"/>
-      <c r="B87" s="57"/>
-      <c r="C87" s="58"/>
+      <c r="B87" s="81"/>
+      <c r="C87" s="82"/>
       <c r="D87" s="26"/>
     </row>
     <row r="88" spans="1:4" ht="14.25">
@@ -3391,54 +3733,12 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B85:C85"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B72:C72"/>
     <mergeCell ref="B75:C75"/>
@@ -3455,12 +3755,54 @@
     <mergeCell ref="B54:C54"/>
     <mergeCell ref="B55:C55"/>
     <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B87:C87"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.67" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup scale="57" orientation="portrait" r:id="rId1"/>
@@ -3516,17 +3858,17 @@
     </row>
     <row r="2" spans="1:24" ht="19.5" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="95" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
+      <c r="I2" s="96"/>
+      <c r="J2" s="96"/>
       <c r="K2" s="4"/>
       <c r="L2" s="5"/>
       <c r="M2" s="4"/>
@@ -3542,15 +3884,15 @@
     </row>
     <row r="3" spans="1:24" ht="19.5">
       <c r="A3" s="1"/>
-      <c r="B3" s="70"/>
-      <c r="C3" s="71"/>
-      <c r="D3" s="71"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="96"/>
       <c r="K3" s="4"/>
       <c r="L3" s="5"/>
       <c r="M3" s="4"/>
@@ -3567,8 +3909,8 @@
     <row r="4" spans="1:24">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="72"/>
-      <c r="D4" s="71"/>
+      <c r="C4" s="98"/>
+      <c r="D4" s="96"/>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
@@ -3589,19 +3931,19 @@
       <c r="V4" s="4"/>
     </row>
     <row r="5" spans="1:24">
-      <c r="A5" s="79" t="s">
+      <c r="A5" s="105" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="79"/>
-      <c r="C5" s="79"/>
-      <c r="D5" s="92" t="s">
+      <c r="B5" s="105"/>
+      <c r="C5" s="105"/>
+      <c r="D5" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="E5" s="92"/>
-      <c r="F5" s="92"/>
-      <c r="G5" s="92"/>
-      <c r="H5" s="92"/>
-      <c r="I5" s="92"/>
+      <c r="E5" s="97"/>
+      <c r="F5" s="97"/>
+      <c r="G5" s="97"/>
+      <c r="H5" s="97"/>
+      <c r="I5" s="97"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
@@ -3617,19 +3959,19 @@
       <c r="V5" s="10"/>
     </row>
     <row r="6" spans="1:24">
-      <c r="A6" s="79" t="s">
+      <c r="A6" s="105" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="79"/>
-      <c r="C6" s="79"/>
-      <c r="D6" s="92" t="s">
+      <c r="B6" s="105"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="92"/>
-      <c r="F6" s="92"/>
-      <c r="G6" s="92"/>
-      <c r="H6" s="92"/>
-      <c r="I6" s="92"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="97"/>
+      <c r="G6" s="97"/>
+      <c r="H6" s="97"/>
+      <c r="I6" s="97"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
@@ -3645,19 +3987,19 @@
       <c r="V6" s="10"/>
     </row>
     <row r="7" spans="1:24">
-      <c r="A7" s="79" t="s">
+      <c r="A7" s="105" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="79"/>
-      <c r="C7" s="79"/>
-      <c r="D7" s="92" t="s">
+      <c r="B7" s="105"/>
+      <c r="C7" s="105"/>
+      <c r="D7" s="97" t="s">
         <v>82</v>
       </c>
-      <c r="E7" s="92"/>
-      <c r="F7" s="92"/>
-      <c r="G7" s="92"/>
-      <c r="H7" s="92"/>
-      <c r="I7" s="92"/>
+      <c r="E7" s="97"/>
+      <c r="F7" s="97"/>
+      <c r="G7" s="97"/>
+      <c r="H7" s="97"/>
+      <c r="I7" s="97"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
@@ -3673,19 +4015,19 @@
       <c r="V7" s="10"/>
     </row>
     <row r="8" spans="1:24">
-      <c r="A8" s="79" t="s">
+      <c r="A8" s="105" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="79"/>
-      <c r="C8" s="79"/>
-      <c r="D8" s="92" t="s">
+      <c r="B8" s="105"/>
+      <c r="C8" s="105"/>
+      <c r="D8" s="97" t="s">
         <v>82</v>
       </c>
-      <c r="E8" s="92"/>
-      <c r="F8" s="92"/>
-      <c r="G8" s="92"/>
-      <c r="H8" s="92"/>
-      <c r="I8" s="92"/>
+      <c r="E8" s="97"/>
+      <c r="F8" s="97"/>
+      <c r="G8" s="97"/>
+      <c r="H8" s="97"/>
+      <c r="I8" s="97"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
@@ -3701,19 +4043,19 @@
       <c r="V8" s="10"/>
     </row>
     <row r="9" spans="1:24">
-      <c r="A9" s="80" t="s">
+      <c r="A9" s="107" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="81"/>
-      <c r="C9" s="82"/>
-      <c r="D9" s="92">
+      <c r="B9" s="108"/>
+      <c r="C9" s="109"/>
+      <c r="D9" s="97">
         <v>3</v>
       </c>
-      <c r="E9" s="92"/>
-      <c r="F9" s="92"/>
-      <c r="G9" s="92"/>
-      <c r="H9" s="92"/>
-      <c r="I9" s="92"/>
+      <c r="E9" s="97"/>
+      <c r="F9" s="97"/>
+      <c r="G9" s="97"/>
+      <c r="H9" s="97"/>
+      <c r="I9" s="97"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
@@ -3729,19 +4071,19 @@
       <c r="V9" s="10"/>
     </row>
     <row r="10" spans="1:24">
-      <c r="A10" s="79" t="s">
+      <c r="A10" s="105" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="79"/>
-      <c r="C10" s="79"/>
-      <c r="D10" s="93">
+      <c r="B10" s="105"/>
+      <c r="C10" s="105"/>
+      <c r="D10" s="106">
         <v>46182</v>
       </c>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
-      <c r="H10" s="93"/>
-      <c r="I10" s="93"/>
+      <c r="E10" s="106"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="106"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
@@ -3761,18 +4103,18 @@
         <v>49</v>
       </c>
       <c r="B11" s="10"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="74"/>
-      <c r="E11" s="75"/>
-      <c r="F11" s="74"/>
-      <c r="G11" s="74"/>
-      <c r="H11" s="74"/>
-      <c r="I11" s="74"/>
-      <c r="J11" s="74"/>
-      <c r="K11" s="74"/>
-      <c r="L11" s="74"/>
-      <c r="M11" s="74"/>
-      <c r="N11" s="74"/>
+      <c r="C11" s="99"/>
+      <c r="D11" s="100"/>
+      <c r="E11" s="101"/>
+      <c r="F11" s="100"/>
+      <c r="G11" s="100"/>
+      <c r="H11" s="100"/>
+      <c r="I11" s="100"/>
+      <c r="J11" s="100"/>
+      <c r="K11" s="100"/>
+      <c r="L11" s="100"/>
+      <c r="M11" s="100"/>
+      <c r="N11" s="100"/>
       <c r="O11" s="10"/>
       <c r="P11" s="10"/>
       <c r="Q11" s="10"/>
@@ -3812,13 +4154,13 @@
       <c r="I12" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="J12" s="76" t="s">
+      <c r="J12" s="102" t="s">
         <v>59</v>
       </c>
-      <c r="K12" s="77"/>
-      <c r="L12" s="77"/>
-      <c r="M12" s="77"/>
-      <c r="N12" s="78"/>
+      <c r="K12" s="103"/>
+      <c r="L12" s="103"/>
+      <c r="M12" s="103"/>
+      <c r="N12" s="104"/>
       <c r="O12" s="14"/>
       <c r="P12" s="14"/>
       <c r="Q12" s="14"/>
@@ -3866,41 +4208,41 @@
       <c r="W13" s="14"/>
       <c r="X13" s="14"/>
     </row>
-    <row r="14" spans="1:24" ht="38.25">
-      <c r="A14" s="94">
+    <row r="14" spans="1:24" ht="38.25" customHeight="1">
+      <c r="A14" s="87">
         <v>1</v>
       </c>
-      <c r="B14" s="95" t="s">
+      <c r="B14" s="88" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="95" t="s">
+      <c r="C14" s="88" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="95" t="s">
+      <c r="D14" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="92">
+      <c r="E14" s="97">
         <v>1</v>
       </c>
-      <c r="F14" s="95" t="s">
+      <c r="F14" s="88" t="s">
         <v>85</v>
       </c>
-      <c r="G14" s="96" t="s">
+      <c r="G14" s="63" t="s">
         <v>86</v>
       </c>
-      <c r="H14" s="96" t="s">
+      <c r="H14" s="63" t="s">
         <v>87</v>
       </c>
-      <c r="I14" s="97" t="s">
+      <c r="I14" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="J14" s="98" t="s">
+      <c r="J14" s="92" t="s">
         <v>89</v>
       </c>
-      <c r="K14" s="98"/>
-      <c r="L14" s="98"/>
-      <c r="M14" s="99"/>
-      <c r="N14" s="95" t="s">
+      <c r="K14" s="92"/>
+      <c r="L14" s="92"/>
+      <c r="M14" s="91"/>
+      <c r="N14" s="88" t="s">
         <v>90</v>
       </c>
       <c r="O14" s="21"/>
@@ -3915,26 +4257,26 @@
       <c r="X14" s="21"/>
     </row>
     <row r="15" spans="1:24" ht="51">
-      <c r="A15" s="94"/>
-      <c r="B15" s="94"/>
-      <c r="C15" s="94"/>
-      <c r="D15" s="94"/>
-      <c r="E15" s="94"/>
-      <c r="F15" s="94"/>
-      <c r="G15" s="100" t="s">
+      <c r="A15" s="87"/>
+      <c r="B15" s="87"/>
+      <c r="C15" s="87"/>
+      <c r="D15" s="87"/>
+      <c r="E15" s="87"/>
+      <c r="F15" s="87"/>
+      <c r="G15" s="65" t="s">
         <v>91</v>
       </c>
-      <c r="H15" s="100" t="s">
+      <c r="H15" s="65" t="s">
         <v>92</v>
       </c>
-      <c r="I15" s="101" t="s">
+      <c r="I15" s="66" t="s">
         <v>93</v>
       </c>
-      <c r="J15" s="98"/>
-      <c r="K15" s="98"/>
-      <c r="L15" s="98"/>
-      <c r="M15" s="98"/>
-      <c r="N15" s="98"/>
+      <c r="J15" s="92"/>
+      <c r="K15" s="92"/>
+      <c r="L15" s="92"/>
+      <c r="M15" s="92"/>
+      <c r="N15" s="92"/>
       <c r="O15" s="21"/>
       <c r="P15" s="21"/>
       <c r="Q15" s="21"/>
@@ -3946,41 +4288,41 @@
       <c r="W15" s="21"/>
       <c r="X15" s="21"/>
     </row>
-    <row r="16" spans="1:24" ht="38.25">
-      <c r="A16" s="102">
+    <row r="16" spans="1:24" ht="38.25" customHeight="1">
+      <c r="A16" s="90">
         <v>1</v>
       </c>
-      <c r="B16" s="103" t="s">
+      <c r="B16" s="86" t="s">
         <v>83</v>
       </c>
-      <c r="C16" s="103" t="s">
+      <c r="C16" s="86" t="s">
         <v>84</v>
       </c>
-      <c r="D16" s="103" t="s">
+      <c r="D16" s="86" t="s">
         <v>65</v>
       </c>
-      <c r="E16" s="102">
+      <c r="E16" s="90">
         <v>2</v>
       </c>
-      <c r="F16" s="103" t="s">
+      <c r="F16" s="86" t="s">
         <v>94</v>
       </c>
-      <c r="G16" s="104" t="s">
+      <c r="G16" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="100" t="s">
+      <c r="H16" s="65" t="s">
         <v>87</v>
       </c>
-      <c r="I16" s="104" t="s">
+      <c r="I16" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="J16" s="105" t="s">
+      <c r="J16" s="93" t="s">
         <v>89</v>
       </c>
-      <c r="K16" s="105"/>
-      <c r="L16" s="105"/>
-      <c r="M16" s="105"/>
-      <c r="N16" s="106" t="s">
+      <c r="K16" s="93"/>
+      <c r="L16" s="93"/>
+      <c r="M16" s="93"/>
+      <c r="N16" s="94" t="s">
         <v>95</v>
       </c>
       <c r="O16" s="21"/>
@@ -3995,26 +4337,26 @@
       <c r="X16" s="21"/>
     </row>
     <row r="17" spans="1:24" ht="25.5" customHeight="1">
-      <c r="A17" s="102"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="102"/>
-      <c r="F17" s="102"/>
-      <c r="G17" s="104" t="s">
+      <c r="A17" s="90"/>
+      <c r="B17" s="90"/>
+      <c r="C17" s="90"/>
+      <c r="D17" s="90"/>
+      <c r="E17" s="90"/>
+      <c r="F17" s="90"/>
+      <c r="G17" s="68" t="s">
         <v>96</v>
       </c>
-      <c r="H17" s="96" t="s">
+      <c r="H17" s="63" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="96" t="s">
+      <c r="I17" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="J17" s="105"/>
-      <c r="K17" s="105"/>
-      <c r="L17" s="105"/>
-      <c r="M17" s="105"/>
-      <c r="N17" s="105"/>
+      <c r="J17" s="93"/>
+      <c r="K17" s="93"/>
+      <c r="L17" s="93"/>
+      <c r="M17" s="93"/>
+      <c r="N17" s="93"/>
       <c r="O17" s="21"/>
       <c r="P17" s="21"/>
       <c r="Q17" s="21"/>
@@ -4026,41 +4368,41 @@
       <c r="W17" s="21"/>
       <c r="X17" s="21"/>
     </row>
-    <row r="18" spans="1:24" ht="51">
-      <c r="A18" s="94">
+    <row r="18" spans="1:24" ht="51" customHeight="1">
+      <c r="A18" s="87">
         <v>2</v>
       </c>
-      <c r="B18" s="103" t="s">
+      <c r="B18" s="86" t="s">
         <v>99</v>
       </c>
-      <c r="C18" s="103" t="s">
+      <c r="C18" s="86" t="s">
         <v>100</v>
       </c>
-      <c r="D18" s="103" t="s">
+      <c r="D18" s="86" t="s">
         <v>65</v>
       </c>
-      <c r="E18" s="102">
+      <c r="E18" s="90">
         <v>1</v>
       </c>
-      <c r="F18" s="103" t="s">
+      <c r="F18" s="86" t="s">
         <v>101</v>
       </c>
-      <c r="G18" s="100" t="s">
+      <c r="G18" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="H18" s="107" t="s">
+      <c r="H18" s="67" t="s">
         <v>103</v>
       </c>
-      <c r="I18" s="96" t="s">
+      <c r="I18" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="94" t="s">
+      <c r="J18" s="87" t="s">
         <v>89</v>
       </c>
-      <c r="K18" s="108"/>
-      <c r="L18" s="108"/>
-      <c r="M18" s="108"/>
-      <c r="N18" s="103" t="s">
+      <c r="K18" s="89"/>
+      <c r="L18" s="89"/>
+      <c r="M18" s="89"/>
+      <c r="N18" s="86" t="s">
         <v>105</v>
       </c>
       <c r="O18" s="21"/>
@@ -4074,27 +4416,27 @@
       <c r="W18" s="21"/>
       <c r="X18" s="21"/>
     </row>
-    <row r="19" spans="1:24" ht="25.5">
-      <c r="A19" s="94"/>
-      <c r="B19" s="94"/>
-      <c r="C19" s="94"/>
-      <c r="D19" s="94"/>
-      <c r="E19" s="94"/>
-      <c r="F19" s="94"/>
-      <c r="G19" s="100" t="s">
+    <row r="19" spans="1:24" ht="38.25" customHeight="1">
+      <c r="A19" s="87"/>
+      <c r="B19" s="87"/>
+      <c r="C19" s="87"/>
+      <c r="D19" s="87"/>
+      <c r="E19" s="87"/>
+      <c r="F19" s="87"/>
+      <c r="G19" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="H19" s="107" t="s">
+      <c r="H19" s="67" t="s">
         <v>107</v>
       </c>
-      <c r="I19" s="96" t="s">
+      <c r="I19" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="J19" s="94"/>
-      <c r="K19" s="94"/>
-      <c r="L19" s="94"/>
-      <c r="M19" s="94"/>
-      <c r="N19" s="94"/>
+      <c r="J19" s="87"/>
+      <c r="K19" s="87"/>
+      <c r="L19" s="87"/>
+      <c r="M19" s="87"/>
+      <c r="N19" s="87"/>
       <c r="O19" s="21"/>
       <c r="P19" s="21"/>
       <c r="Q19" s="21"/>
@@ -4107,636 +4449,1068 @@
       <c r="X19" s="21"/>
     </row>
     <row r="20" spans="1:24" ht="38.25">
-      <c r="A20" s="94"/>
-      <c r="B20" s="94"/>
-      <c r="C20" s="94"/>
-      <c r="D20" s="94"/>
-      <c r="E20" s="94"/>
-      <c r="F20" s="94"/>
-      <c r="G20" s="109" t="s">
+      <c r="A20" s="87"/>
+      <c r="B20" s="87"/>
+      <c r="C20" s="87"/>
+      <c r="D20" s="87"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="H20" s="109" t="s">
+      <c r="H20" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="I20" s="109" t="s">
+      <c r="I20" s="62" t="s">
         <v>110</v>
       </c>
-      <c r="J20" s="94"/>
-      <c r="K20" s="94"/>
-      <c r="L20" s="94"/>
-      <c r="M20" s="94"/>
-      <c r="N20" s="94"/>
-    </row>
-    <row r="21" spans="1:24" ht="25.5">
-      <c r="A21" s="94">
+      <c r="J20" s="87"/>
+      <c r="K20" s="87"/>
+      <c r="L20" s="87"/>
+      <c r="M20" s="87"/>
+      <c r="N20" s="87"/>
+    </row>
+    <row r="21" spans="1:24" ht="25.5" customHeight="1">
+      <c r="A21" s="87">
         <v>3</v>
       </c>
-      <c r="B21" s="95" t="s">
+      <c r="B21" s="88" t="s">
         <v>111</v>
       </c>
-      <c r="C21" s="95" t="s">
+      <c r="C21" s="88" t="s">
         <v>112</v>
       </c>
-      <c r="D21" s="95" t="s">
+      <c r="D21" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="94">
+      <c r="E21" s="87">
         <v>1</v>
       </c>
-      <c r="F21" s="95" t="s">
+      <c r="F21" s="88" t="s">
         <v>113</v>
       </c>
-      <c r="G21" s="109" t="s">
+      <c r="G21" s="62" t="s">
         <v>114</v>
       </c>
-      <c r="H21" s="109" t="s">
+      <c r="H21" s="62" t="s">
         <v>115</v>
       </c>
-      <c r="I21" s="109" t="s">
+      <c r="I21" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="J21" s="94" t="s">
+      <c r="J21" s="87" t="s">
         <v>89</v>
       </c>
-      <c r="K21" s="108"/>
-      <c r="L21" s="108"/>
-      <c r="M21" s="108"/>
-      <c r="N21" s="103" t="s">
+      <c r="K21" s="89"/>
+      <c r="L21" s="89"/>
+      <c r="M21" s="89"/>
+      <c r="N21" s="86" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="38.25">
-      <c r="A22" s="94"/>
-      <c r="B22" s="94"/>
-      <c r="C22" s="94"/>
-      <c r="D22" s="94"/>
-      <c r="E22" s="94"/>
-      <c r="F22" s="94"/>
-      <c r="G22" s="109" t="s">
+    <row r="22" spans="1:24" ht="38.25" customHeight="1">
+      <c r="A22" s="87"/>
+      <c r="B22" s="87"/>
+      <c r="C22" s="87"/>
+      <c r="D22" s="87"/>
+      <c r="E22" s="87"/>
+      <c r="F22" s="87"/>
+      <c r="G22" s="62" t="s">
         <v>118</v>
       </c>
-      <c r="H22" s="109" t="s">
+      <c r="H22" s="62" t="s">
         <v>119</v>
       </c>
-      <c r="I22" s="109" t="s">
+      <c r="I22" s="62" t="s">
         <v>120</v>
       </c>
-      <c r="J22" s="94"/>
-      <c r="K22" s="94"/>
-      <c r="L22" s="94"/>
-      <c r="M22" s="94"/>
-      <c r="N22" s="94"/>
+      <c r="J22" s="87"/>
+      <c r="K22" s="87"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="87"/>
+      <c r="N22" s="87"/>
     </row>
     <row r="23" spans="1:24" ht="38.25">
-      <c r="A23" s="94"/>
-      <c r="B23" s="94"/>
-      <c r="C23" s="94"/>
-      <c r="D23" s="94"/>
-      <c r="E23" s="94"/>
-      <c r="F23" s="94"/>
-      <c r="G23" s="109" t="s">
+      <c r="A23" s="87"/>
+      <c r="B23" s="87"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="87"/>
+      <c r="E23" s="87"/>
+      <c r="F23" s="87"/>
+      <c r="G23" s="62" t="s">
         <v>121</v>
       </c>
-      <c r="H23" s="109" t="s">
+      <c r="H23" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="I23" s="109" t="s">
+      <c r="I23" s="62" t="s">
         <v>122</v>
       </c>
-      <c r="J23" s="94"/>
-      <c r="K23" s="94"/>
-      <c r="L23" s="94"/>
-      <c r="M23" s="94"/>
-      <c r="N23" s="94"/>
-    </row>
-    <row r="24" spans="1:24" ht="25.5">
-      <c r="A24" s="94">
+      <c r="J23" s="87"/>
+      <c r="K23" s="87"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="87"/>
+      <c r="N23" s="87"/>
+    </row>
+    <row r="24" spans="1:24" ht="25.5" customHeight="1">
+      <c r="A24" s="87">
         <v>4</v>
       </c>
-      <c r="B24" s="95" t="s">
+      <c r="B24" s="88" t="s">
         <v>123</v>
       </c>
-      <c r="C24" s="95" t="s">
+      <c r="C24" s="88" t="s">
         <v>124</v>
       </c>
-      <c r="D24" s="95" t="s">
+      <c r="D24" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="E24" s="94">
+      <c r="E24" s="87">
         <v>1</v>
       </c>
-      <c r="F24" s="95" t="s">
+      <c r="F24" s="88" t="s">
         <v>125</v>
       </c>
-      <c r="G24" s="109" t="s">
+      <c r="G24" s="62" t="s">
         <v>126</v>
       </c>
-      <c r="H24" s="109" t="s">
+      <c r="H24" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="I24" s="109" t="s">
+      <c r="I24" s="62" t="s">
         <v>128</v>
       </c>
-      <c r="J24" s="94" t="s">
+      <c r="J24" s="87" t="s">
         <v>89</v>
       </c>
-      <c r="K24" s="108"/>
-      <c r="L24" s="108"/>
-      <c r="M24" s="108"/>
-      <c r="N24" s="103" t="s">
+      <c r="K24" s="89"/>
+      <c r="L24" s="89"/>
+      <c r="M24" s="89"/>
+      <c r="N24" s="86" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="25.5">
-      <c r="A25" s="94"/>
-      <c r="B25" s="94"/>
-      <c r="C25" s="94"/>
-      <c r="D25" s="94"/>
-      <c r="E25" s="94"/>
-      <c r="F25" s="94"/>
-      <c r="G25" s="109" t="s">
+    <row r="25" spans="1:24" ht="38.25" customHeight="1">
+      <c r="A25" s="87"/>
+      <c r="B25" s="87"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="87"/>
+      <c r="F25" s="87"/>
+      <c r="G25" s="62" t="s">
         <v>130</v>
       </c>
-      <c r="H25" s="109" t="s">
+      <c r="H25" s="62" t="s">
         <v>131</v>
       </c>
-      <c r="I25" s="109" t="s">
+      <c r="I25" s="62" t="s">
         <v>132</v>
       </c>
-      <c r="J25" s="94"/>
-      <c r="K25" s="94"/>
-      <c r="L25" s="94"/>
-      <c r="M25" s="94"/>
-      <c r="N25" s="94"/>
-    </row>
-    <row r="26" spans="1:24" ht="38.25">
-      <c r="A26" s="94"/>
-      <c r="B26" s="94"/>
-      <c r="C26" s="94"/>
-      <c r="D26" s="94"/>
-      <c r="E26" s="94"/>
-      <c r="F26" s="94"/>
-      <c r="G26" s="109" t="s">
+      <c r="J25" s="87"/>
+      <c r="K25" s="87"/>
+      <c r="L25" s="87"/>
+      <c r="M25" s="87"/>
+      <c r="N25" s="87"/>
+    </row>
+    <row r="26" spans="1:24" ht="38.25" customHeight="1">
+      <c r="A26" s="87"/>
+      <c r="B26" s="87"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="87"/>
+      <c r="E26" s="87"/>
+      <c r="F26" s="87"/>
+      <c r="G26" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="H26" s="109" t="s">
+      <c r="H26" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="I26" s="109" t="s">
+      <c r="I26" s="62" t="s">
         <v>134</v>
       </c>
-      <c r="J26" s="94"/>
-      <c r="K26" s="94"/>
-      <c r="L26" s="94"/>
-      <c r="M26" s="94"/>
-      <c r="N26" s="94"/>
-    </row>
-    <row r="27" spans="1:24" ht="38.25">
-      <c r="A27" s="94">
+      <c r="J26" s="87"/>
+      <c r="K26" s="87"/>
+      <c r="L26" s="87"/>
+      <c r="M26" s="87"/>
+      <c r="N26" s="87"/>
+    </row>
+    <row r="27" spans="1:24" ht="38.25" customHeight="1">
+      <c r="A27" s="87">
         <v>5</v>
       </c>
-      <c r="B27" s="95" t="s">
+      <c r="B27" s="88" t="s">
         <v>135</v>
       </c>
-      <c r="C27" s="95" t="s">
+      <c r="C27" s="88" t="s">
         <v>136</v>
       </c>
-      <c r="D27" s="95" t="s">
+      <c r="D27" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="94">
+      <c r="E27" s="87">
         <v>1</v>
       </c>
-      <c r="F27" s="95" t="s">
+      <c r="F27" s="88" t="s">
         <v>137</v>
       </c>
-      <c r="G27" s="109" t="s">
+      <c r="G27" s="62" t="s">
         <v>138</v>
       </c>
-      <c r="H27" s="109" t="s">
+      <c r="H27" s="62" t="s">
         <v>139</v>
       </c>
-      <c r="I27" s="109" t="s">
+      <c r="I27" s="62" t="s">
         <v>140</v>
       </c>
-      <c r="J27" s="94" t="s">
+      <c r="J27" s="87" t="s">
         <v>89</v>
       </c>
-      <c r="K27" s="108"/>
-      <c r="L27" s="108"/>
-      <c r="M27" s="108"/>
-      <c r="N27" s="103" t="s">
+      <c r="K27" s="89"/>
+      <c r="L27" s="89"/>
+      <c r="M27" s="89"/>
+      <c r="N27" s="86" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:24" ht="25.5">
-      <c r="A28" s="94"/>
-      <c r="B28" s="94"/>
-      <c r="C28" s="94"/>
-      <c r="D28" s="94"/>
-      <c r="E28" s="94"/>
-      <c r="F28" s="94"/>
-      <c r="G28" s="109" t="s">
+      <c r="A28" s="87"/>
+      <c r="B28" s="87"/>
+      <c r="C28" s="87"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="87"/>
+      <c r="F28" s="87"/>
+      <c r="G28" s="62" t="s">
         <v>142</v>
       </c>
-      <c r="H28" s="109" t="s">
+      <c r="H28" s="62" t="s">
         <v>143</v>
       </c>
-      <c r="I28" s="109" t="s">
+      <c r="I28" s="62" t="s">
         <v>144</v>
       </c>
-      <c r="J28" s="94"/>
-      <c r="K28" s="94"/>
-      <c r="L28" s="94"/>
-      <c r="M28" s="94"/>
-      <c r="N28" s="94"/>
-    </row>
-    <row r="29" spans="1:24" ht="25.5">
-      <c r="A29" s="94">
+      <c r="J28" s="87"/>
+      <c r="K28" s="87"/>
+      <c r="L28" s="87"/>
+      <c r="M28" s="87"/>
+      <c r="N28" s="87"/>
+    </row>
+    <row r="29" spans="1:24" ht="25.5" customHeight="1">
+      <c r="A29" s="87">
         <v>6</v>
       </c>
-      <c r="B29" s="95" t="s">
+      <c r="B29" s="88" t="s">
         <v>145</v>
       </c>
-      <c r="C29" s="95" t="s">
+      <c r="C29" s="88" t="s">
         <v>146</v>
       </c>
-      <c r="D29" s="95" t="s">
+      <c r="D29" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="94">
+      <c r="E29" s="87">
         <v>1</v>
       </c>
-      <c r="F29" s="95" t="s">
+      <c r="F29" s="88" t="s">
         <v>147</v>
       </c>
-      <c r="G29" s="109" t="s">
+      <c r="G29" s="62" t="s">
         <v>148</v>
       </c>
-      <c r="H29" s="109" t="s">
+      <c r="H29" s="62" t="s">
         <v>149</v>
       </c>
-      <c r="I29" s="109" t="s">
+      <c r="I29" s="62" t="s">
         <v>150</v>
       </c>
-      <c r="J29" s="94" t="s">
+      <c r="J29" s="87" t="s">
         <v>89</v>
       </c>
-      <c r="K29" s="108"/>
-      <c r="L29" s="108"/>
-      <c r="M29" s="108"/>
-      <c r="N29" s="103" t="s">
+      <c r="K29" s="89"/>
+      <c r="L29" s="89"/>
+      <c r="M29" s="89"/>
+      <c r="N29" s="86" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="30" spans="1:24" ht="51">
-      <c r="A30" s="94"/>
-      <c r="B30" s="94"/>
-      <c r="C30" s="94"/>
-      <c r="D30" s="94"/>
-      <c r="E30" s="94"/>
-      <c r="F30" s="94"/>
-      <c r="G30" s="109" t="s">
+      <c r="A30" s="87"/>
+      <c r="B30" s="87"/>
+      <c r="C30" s="87"/>
+      <c r="D30" s="87"/>
+      <c r="E30" s="87"/>
+      <c r="F30" s="87"/>
+      <c r="G30" s="62" t="s">
         <v>152</v>
       </c>
-      <c r="H30" s="109" t="s">
+      <c r="H30" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="I30" s="109" t="s">
+      <c r="I30" s="62" t="s">
         <v>153</v>
       </c>
-      <c r="J30" s="94"/>
-      <c r="K30" s="94"/>
-      <c r="L30" s="94"/>
-      <c r="M30" s="94"/>
-      <c r="N30" s="94"/>
-    </row>
-    <row r="31" spans="1:24">
-      <c r="A31" s="21"/>
-      <c r="B31" s="21"/>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-    </row>
-    <row r="32" spans="1:24">
-      <c r="A32" s="21"/>
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-    </row>
-    <row r="33" spans="1:10">
-      <c r="A33" s="21"/>
-      <c r="B33" s="21"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-    </row>
-    <row r="34" spans="1:10">
-      <c r="A34" s="21"/>
-      <c r="B34" s="21"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="21"/>
-      <c r="I34" s="21"/>
-      <c r="J34" s="21"/>
-    </row>
-    <row r="35" spans="1:10">
-      <c r="A35" s="21"/>
-      <c r="B35" s="21"/>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="21"/>
-      <c r="H35" s="21"/>
-      <c r="I35" s="21"/>
-      <c r="J35" s="21"/>
-    </row>
-    <row r="36" spans="1:10">
-      <c r="A36" s="21"/>
-      <c r="B36" s="21"/>
-      <c r="C36" s="21"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="21"/>
-      <c r="J36" s="21"/>
-    </row>
-    <row r="37" spans="1:10">
-      <c r="A37" s="21"/>
-      <c r="B37" s="21"/>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
-      <c r="G37" s="21"/>
-      <c r="H37" s="21"/>
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
-    </row>
-    <row r="38" spans="1:10">
-      <c r="A38" s="21"/>
-      <c r="B38" s="21"/>
-      <c r="C38" s="21"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
-      <c r="G38" s="21"/>
-      <c r="H38" s="21"/>
-      <c r="I38" s="21"/>
-      <c r="J38" s="21"/>
-    </row>
-    <row r="39" spans="1:10">
-      <c r="A39" s="21"/>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
-      <c r="H39" s="21"/>
-      <c r="I39" s="21"/>
-      <c r="J39" s="21"/>
-    </row>
-    <row r="40" spans="1:10">
-      <c r="A40" s="21"/>
-      <c r="B40" s="21"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
-      <c r="H40" s="21"/>
-      <c r="I40" s="21"/>
-      <c r="J40" s="21"/>
-    </row>
-    <row r="41" spans="1:10">
-      <c r="A41" s="21"/>
-      <c r="B41" s="21"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="21"/>
-      <c r="J41" s="21"/>
-    </row>
-    <row r="42" spans="1:10">
-      <c r="A42" s="21"/>
-      <c r="B42" s="21"/>
-      <c r="C42" s="21"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21"/>
-      <c r="G42" s="21"/>
-      <c r="H42" s="21"/>
-      <c r="I42" s="21"/>
-      <c r="J42" s="21"/>
-    </row>
-    <row r="43" spans="1:10">
-      <c r="A43" s="21"/>
-      <c r="B43" s="21"/>
-      <c r="C43" s="21"/>
-      <c r="D43" s="21"/>
-      <c r="E43" s="21"/>
-      <c r="F43" s="21"/>
-      <c r="G43" s="21"/>
-      <c r="H43" s="21"/>
-      <c r="I43" s="21"/>
-      <c r="J43" s="21"/>
-    </row>
-    <row r="44" spans="1:10">
-      <c r="A44" s="21"/>
-      <c r="B44" s="21"/>
-      <c r="C44" s="21"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="21"/>
-      <c r="F44" s="21"/>
-      <c r="G44" s="21"/>
-      <c r="H44" s="21"/>
-      <c r="I44" s="21"/>
-      <c r="J44" s="21"/>
-    </row>
-    <row r="45" spans="1:10">
-      <c r="A45" s="21"/>
-      <c r="B45" s="21"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
-      <c r="F45" s="21"/>
-      <c r="G45" s="21"/>
-      <c r="H45" s="21"/>
-      <c r="I45" s="21"/>
-      <c r="J45" s="21"/>
-    </row>
-    <row r="46" spans="1:10">
-      <c r="A46" s="21"/>
-      <c r="B46" s="21"/>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
-      <c r="H46" s="21"/>
-      <c r="I46" s="21"/>
-      <c r="J46" s="21"/>
-    </row>
-    <row r="47" spans="1:10">
-      <c r="A47" s="21"/>
-      <c r="B47" s="21"/>
-      <c r="C47" s="21"/>
-      <c r="D47" s="21"/>
-      <c r="E47" s="21"/>
-      <c r="F47" s="21"/>
-      <c r="G47" s="21"/>
-      <c r="H47" s="21"/>
-      <c r="I47" s="21"/>
-      <c r="J47" s="21"/>
-    </row>
-    <row r="48" spans="1:10">
-      <c r="A48" s="21"/>
-      <c r="B48" s="21"/>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
-      <c r="H48" s="21"/>
-      <c r="I48" s="21"/>
-      <c r="J48" s="21"/>
-    </row>
-    <row r="49" spans="1:10">
-      <c r="A49" s="21"/>
-      <c r="B49" s="21"/>
-      <c r="C49" s="21"/>
-      <c r="D49" s="21"/>
-      <c r="E49" s="21"/>
-      <c r="F49" s="21"/>
-      <c r="G49" s="21"/>
-      <c r="H49" s="21"/>
-      <c r="I49" s="21"/>
-      <c r="J49" s="21"/>
-    </row>
-    <row r="50" spans="1:10">
-      <c r="A50" s="21"/>
-      <c r="B50" s="21"/>
-      <c r="C50" s="21"/>
-      <c r="D50" s="21"/>
-      <c r="E50" s="21"/>
-      <c r="F50" s="21"/>
-      <c r="G50" s="21"/>
-      <c r="H50" s="21"/>
-      <c r="I50" s="21"/>
-      <c r="J50" s="21"/>
-    </row>
-    <row r="51" spans="1:10">
-      <c r="A51" s="21"/>
-      <c r="B51" s="21"/>
-      <c r="C51" s="21"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="21"/>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
-      <c r="H51" s="21"/>
-      <c r="I51" s="21"/>
-      <c r="J51" s="21"/>
-    </row>
-    <row r="52" spans="1:10">
-      <c r="A52" s="21"/>
-      <c r="B52" s="21"/>
-      <c r="C52" s="21"/>
-      <c r="D52" s="21"/>
-      <c r="E52" s="21"/>
-      <c r="F52" s="21"/>
-      <c r="G52" s="21"/>
-      <c r="H52" s="21"/>
-      <c r="I52" s="21"/>
-      <c r="J52" s="21"/>
-    </row>
-    <row r="53" spans="1:10">
-      <c r="A53" s="21"/>
-      <c r="B53" s="21"/>
-      <c r="C53" s="21"/>
-      <c r="D53" s="21"/>
-      <c r="E53" s="21"/>
-      <c r="F53" s="21"/>
-      <c r="G53" s="21"/>
-      <c r="H53" s="21"/>
-      <c r="I53" s="21"/>
-      <c r="J53" s="21"/>
-    </row>
-    <row r="54" spans="1:10">
-      <c r="A54" s="21"/>
-      <c r="B54" s="21"/>
-      <c r="C54" s="21"/>
-      <c r="D54" s="21"/>
-      <c r="E54" s="21"/>
-      <c r="F54" s="21"/>
-      <c r="G54" s="21"/>
-      <c r="H54" s="21"/>
-      <c r="I54" s="21"/>
-      <c r="J54" s="21"/>
-    </row>
-    <row r="55" spans="1:10">
-      <c r="A55" s="21"/>
-      <c r="B55" s="21"/>
-      <c r="C55" s="21"/>
-      <c r="D55" s="21"/>
-      <c r="E55" s="21"/>
-      <c r="F55" s="21"/>
-      <c r="G55" s="21"/>
-      <c r="H55" s="21"/>
-      <c r="I55" s="21"/>
-      <c r="J55" s="21"/>
-    </row>
-    <row r="56" spans="1:10">
-      <c r="A56" s="21"/>
-      <c r="B56" s="21"/>
-      <c r="C56" s="21"/>
-      <c r="D56" s="21"/>
-      <c r="E56" s="21"/>
-      <c r="F56" s="21"/>
-      <c r="G56" s="21"/>
-      <c r="H56" s="21"/>
-      <c r="I56" s="21"/>
-      <c r="J56" s="21"/>
-    </row>
-    <row r="57" spans="1:10">
-      <c r="A57" s="21"/>
-      <c r="B57" s="21"/>
-      <c r="C57" s="21"/>
-      <c r="D57" s="21"/>
-      <c r="E57" s="21"/>
-      <c r="F57" s="21"/>
-      <c r="G57" s="21"/>
-      <c r="H57" s="21"/>
-      <c r="I57" s="21"/>
-      <c r="J57" s="21"/>
-    </row>
-    <row r="58" spans="1:10">
+      <c r="J30" s="87"/>
+      <c r="K30" s="87"/>
+      <c r="L30" s="87"/>
+      <c r="M30" s="87"/>
+      <c r="N30" s="87"/>
+    </row>
+    <row r="31" spans="1:24" ht="102" customHeight="1">
+      <c r="A31" s="87">
+        <v>7</v>
+      </c>
+      <c r="B31" s="88" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" s="88" t="s">
+        <v>124</v>
+      </c>
+      <c r="D31" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" s="87">
+        <v>1</v>
+      </c>
+      <c r="F31" s="88" t="s">
+        <v>155</v>
+      </c>
+      <c r="G31" s="62" t="s">
+        <v>156</v>
+      </c>
+      <c r="H31" s="62" t="s">
+        <v>157</v>
+      </c>
+      <c r="I31" s="62" t="s">
+        <v>158</v>
+      </c>
+      <c r="J31" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K31" s="89"/>
+      <c r="L31" s="89"/>
+      <c r="M31" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N31" s="86" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" ht="38.25">
+      <c r="A32" s="87"/>
+      <c r="B32" s="87"/>
+      <c r="C32" s="87"/>
+      <c r="D32" s="87"/>
+      <c r="E32" s="87"/>
+      <c r="F32" s="87"/>
+      <c r="G32" s="62" t="s">
+        <v>159</v>
+      </c>
+      <c r="H32" s="62" t="s">
+        <v>143</v>
+      </c>
+      <c r="I32" s="62" t="s">
+        <v>160</v>
+      </c>
+      <c r="J32" s="87"/>
+      <c r="K32" s="91"/>
+      <c r="L32" s="91"/>
+      <c r="M32" s="91"/>
+      <c r="N32" s="88"/>
+    </row>
+    <row r="33" spans="1:14" ht="25.5" customHeight="1">
+      <c r="A33" s="87"/>
+      <c r="B33" s="87"/>
+      <c r="C33" s="87"/>
+      <c r="D33" s="87"/>
+      <c r="E33" s="87"/>
+      <c r="F33" s="87"/>
+      <c r="G33" s="62" t="s">
+        <v>161</v>
+      </c>
+      <c r="H33" s="62" t="s">
+        <v>162</v>
+      </c>
+      <c r="I33" s="62" t="s">
+        <v>163</v>
+      </c>
+      <c r="J33" s="87"/>
+      <c r="K33" s="91"/>
+      <c r="L33" s="91"/>
+      <c r="M33" s="91"/>
+      <c r="N33" s="88"/>
+    </row>
+    <row r="34" spans="1:14" ht="76.5" customHeight="1">
+      <c r="A34" s="87">
+        <v>8</v>
+      </c>
+      <c r="B34" s="88" t="s">
+        <v>164</v>
+      </c>
+      <c r="C34" s="88" t="s">
+        <v>84</v>
+      </c>
+      <c r="D34" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="87">
+        <v>1</v>
+      </c>
+      <c r="F34" s="88" t="s">
+        <v>165</v>
+      </c>
+      <c r="G34" s="62" t="s">
+        <v>166</v>
+      </c>
+      <c r="H34" s="62" t="s">
+        <v>167</v>
+      </c>
+      <c r="I34" s="62" t="s">
+        <v>88</v>
+      </c>
+      <c r="J34" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K34" s="89"/>
+      <c r="L34" s="89"/>
+      <c r="M34" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N34" s="110" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="63.75">
+      <c r="A35" s="87"/>
+      <c r="B35" s="87"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="87"/>
+      <c r="E35" s="87"/>
+      <c r="F35" s="87"/>
+      <c r="G35" s="62" t="s">
+        <v>168</v>
+      </c>
+      <c r="H35" s="62" t="s">
+        <v>169</v>
+      </c>
+      <c r="I35" s="62" t="s">
+        <v>170</v>
+      </c>
+      <c r="J35" s="87"/>
+      <c r="K35" s="91"/>
+      <c r="L35" s="91"/>
+      <c r="M35" s="91"/>
+      <c r="N35" s="88"/>
+    </row>
+    <row r="36" spans="1:14" ht="89.25" customHeight="1">
+      <c r="A36" s="87">
+        <v>9</v>
+      </c>
+      <c r="B36" s="88" t="s">
+        <v>171</v>
+      </c>
+      <c r="C36" s="88" t="s">
+        <v>84</v>
+      </c>
+      <c r="D36" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="E36" s="87">
+        <v>1</v>
+      </c>
+      <c r="F36" s="88" t="s">
+        <v>172</v>
+      </c>
+      <c r="G36" s="62" t="s">
+        <v>173</v>
+      </c>
+      <c r="H36" s="62" t="s">
+        <v>174</v>
+      </c>
+      <c r="I36" s="62" t="s">
+        <v>175</v>
+      </c>
+      <c r="J36" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K36" s="89"/>
+      <c r="L36" s="89"/>
+      <c r="M36" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N36" s="110" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="38.25">
+      <c r="A37" s="87"/>
+      <c r="B37" s="87"/>
+      <c r="C37" s="87"/>
+      <c r="D37" s="87"/>
+      <c r="E37" s="87"/>
+      <c r="F37" s="87"/>
+      <c r="G37" s="62" t="s">
+        <v>176</v>
+      </c>
+      <c r="H37" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I37" s="62" t="s">
+        <v>177</v>
+      </c>
+      <c r="J37" s="87"/>
+      <c r="K37" s="91"/>
+      <c r="L37" s="91"/>
+      <c r="M37" s="91"/>
+      <c r="N37" s="88"/>
+    </row>
+    <row r="38" spans="1:14" ht="38.25" customHeight="1">
+      <c r="A38" s="87"/>
+      <c r="B38" s="87"/>
+      <c r="C38" s="87"/>
+      <c r="D38" s="87"/>
+      <c r="E38" s="87"/>
+      <c r="F38" s="87"/>
+      <c r="G38" s="62" t="s">
+        <v>178</v>
+      </c>
+      <c r="H38" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I38" s="62" t="s">
+        <v>179</v>
+      </c>
+      <c r="J38" s="87"/>
+      <c r="K38" s="91"/>
+      <c r="L38" s="91"/>
+      <c r="M38" s="91"/>
+      <c r="N38" s="88"/>
+    </row>
+    <row r="39" spans="1:14" ht="76.5" customHeight="1">
+      <c r="A39" s="87">
+        <v>10</v>
+      </c>
+      <c r="B39" s="88" t="s">
+        <v>180</v>
+      </c>
+      <c r="C39" s="88" t="s">
+        <v>181</v>
+      </c>
+      <c r="D39" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="E39" s="87">
+        <v>1</v>
+      </c>
+      <c r="F39" s="88" t="s">
+        <v>182</v>
+      </c>
+      <c r="G39" s="62" t="s">
+        <v>183</v>
+      </c>
+      <c r="H39" s="62" t="s">
+        <v>184</v>
+      </c>
+      <c r="I39" s="62" t="s">
+        <v>185</v>
+      </c>
+      <c r="J39" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K39" s="89"/>
+      <c r="L39" s="89"/>
+      <c r="M39" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N39" s="110" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="25.5">
+      <c r="A40" s="87"/>
+      <c r="B40" s="87"/>
+      <c r="C40" s="87"/>
+      <c r="D40" s="87"/>
+      <c r="E40" s="87"/>
+      <c r="F40" s="87"/>
+      <c r="G40" s="62" t="s">
+        <v>186</v>
+      </c>
+      <c r="H40" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I40" s="62" t="s">
+        <v>187</v>
+      </c>
+      <c r="J40" s="87"/>
+      <c r="K40" s="91"/>
+      <c r="L40" s="91"/>
+      <c r="M40" s="91"/>
+      <c r="N40" s="88"/>
+    </row>
+    <row r="41" spans="1:14" ht="25.5">
+      <c r="A41" s="87"/>
+      <c r="B41" s="87"/>
+      <c r="C41" s="87"/>
+      <c r="D41" s="87"/>
+      <c r="E41" s="87"/>
+      <c r="F41" s="87"/>
+      <c r="G41" s="62" t="s">
+        <v>188</v>
+      </c>
+      <c r="H41" s="62" t="s">
+        <v>189</v>
+      </c>
+      <c r="I41" s="62" t="s">
+        <v>190</v>
+      </c>
+      <c r="J41" s="87"/>
+      <c r="K41" s="91"/>
+      <c r="L41" s="91"/>
+      <c r="M41" s="91"/>
+      <c r="N41" s="88"/>
+    </row>
+    <row r="42" spans="1:14" ht="38.25" customHeight="1">
+      <c r="A42" s="87"/>
+      <c r="B42" s="87"/>
+      <c r="C42" s="87"/>
+      <c r="D42" s="87"/>
+      <c r="E42" s="87"/>
+      <c r="F42" s="87"/>
+      <c r="G42" s="62" t="s">
+        <v>191</v>
+      </c>
+      <c r="H42" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I42" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="J42" s="87"/>
+      <c r="K42" s="91"/>
+      <c r="L42" s="91"/>
+      <c r="M42" s="91"/>
+      <c r="N42" s="88"/>
+    </row>
+    <row r="43" spans="1:14" ht="38.25">
+      <c r="A43" s="87">
+        <v>11</v>
+      </c>
+      <c r="B43" s="88" t="s">
+        <v>193</v>
+      </c>
+      <c r="C43" s="88" t="s">
+        <v>100</v>
+      </c>
+      <c r="D43" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="E43" s="87">
+        <v>1</v>
+      </c>
+      <c r="F43" s="88" t="s">
+        <v>194</v>
+      </c>
+      <c r="G43" s="62" t="s">
+        <v>195</v>
+      </c>
+      <c r="H43" s="62" t="s">
+        <v>196</v>
+      </c>
+      <c r="I43" s="62" t="s">
+        <v>197</v>
+      </c>
+      <c r="J43" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K43" s="89"/>
+      <c r="L43" s="89"/>
+      <c r="M43" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N43" s="110" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="25.5">
+      <c r="A44" s="87"/>
+      <c r="B44" s="87"/>
+      <c r="C44" s="87"/>
+      <c r="D44" s="87"/>
+      <c r="E44" s="87"/>
+      <c r="F44" s="87"/>
+      <c r="G44" s="62" t="s">
+        <v>198</v>
+      </c>
+      <c r="H44" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I44" s="62" t="s">
+        <v>199</v>
+      </c>
+      <c r="J44" s="87"/>
+      <c r="K44" s="91"/>
+      <c r="L44" s="91"/>
+      <c r="M44" s="91"/>
+      <c r="N44" s="88"/>
+    </row>
+    <row r="45" spans="1:14" ht="25.5">
+      <c r="A45" s="87"/>
+      <c r="B45" s="87"/>
+      <c r="C45" s="87"/>
+      <c r="D45" s="87"/>
+      <c r="E45" s="87"/>
+      <c r="F45" s="87"/>
+      <c r="G45" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="H45" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I45" s="62" t="s">
+        <v>201</v>
+      </c>
+      <c r="J45" s="87"/>
+      <c r="K45" s="91"/>
+      <c r="L45" s="91"/>
+      <c r="M45" s="91"/>
+      <c r="N45" s="88"/>
+    </row>
+    <row r="46" spans="1:14" ht="63.75" customHeight="1">
+      <c r="A46" s="87">
+        <v>12</v>
+      </c>
+      <c r="B46" s="88" t="s">
+        <v>202</v>
+      </c>
+      <c r="C46" s="88" t="s">
+        <v>146</v>
+      </c>
+      <c r="D46" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="E46" s="87">
+        <v>1</v>
+      </c>
+      <c r="F46" s="88" t="s">
+        <v>203</v>
+      </c>
+      <c r="G46" s="62" t="s">
+        <v>204</v>
+      </c>
+      <c r="H46" s="62" t="s">
+        <v>205</v>
+      </c>
+      <c r="I46" s="62" t="s">
+        <v>206</v>
+      </c>
+      <c r="J46" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K46" s="89"/>
+      <c r="L46" s="89"/>
+      <c r="M46" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N46" s="110" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="38.25">
+      <c r="A47" s="87"/>
+      <c r="B47" s="87"/>
+      <c r="C47" s="87"/>
+      <c r="D47" s="87"/>
+      <c r="E47" s="87"/>
+      <c r="F47" s="87"/>
+      <c r="G47" s="62" t="s">
+        <v>207</v>
+      </c>
+      <c r="H47" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I47" s="62" t="s">
+        <v>208</v>
+      </c>
+      <c r="J47" s="87"/>
+      <c r="K47" s="91"/>
+      <c r="L47" s="91"/>
+      <c r="M47" s="91"/>
+      <c r="N47" s="88"/>
+    </row>
+    <row r="48" spans="1:14" ht="25.5">
+      <c r="A48" s="87"/>
+      <c r="B48" s="87"/>
+      <c r="C48" s="87"/>
+      <c r="D48" s="87"/>
+      <c r="E48" s="87"/>
+      <c r="F48" s="87"/>
+      <c r="G48" s="62" t="s">
+        <v>209</v>
+      </c>
+      <c r="H48" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I48" s="62" t="s">
+        <v>210</v>
+      </c>
+      <c r="J48" s="87"/>
+      <c r="K48" s="91"/>
+      <c r="L48" s="91"/>
+      <c r="M48" s="91"/>
+      <c r="N48" s="88"/>
+    </row>
+    <row r="49" spans="1:14" ht="25.5">
+      <c r="A49" s="87"/>
+      <c r="B49" s="87"/>
+      <c r="C49" s="87"/>
+      <c r="D49" s="87"/>
+      <c r="E49" s="87"/>
+      <c r="F49" s="87"/>
+      <c r="G49" s="62" t="s">
+        <v>211</v>
+      </c>
+      <c r="H49" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I49" s="62" t="s">
+        <v>212</v>
+      </c>
+      <c r="J49" s="87"/>
+      <c r="K49" s="91"/>
+      <c r="L49" s="91"/>
+      <c r="M49" s="91"/>
+      <c r="N49" s="88"/>
+    </row>
+    <row r="50" spans="1:14" ht="140.25" customHeight="1">
+      <c r="A50" s="87">
+        <v>13</v>
+      </c>
+      <c r="B50" s="88" t="s">
+        <v>213</v>
+      </c>
+      <c r="C50" s="88" t="s">
+        <v>136</v>
+      </c>
+      <c r="D50" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="E50" s="87">
+        <v>1</v>
+      </c>
+      <c r="F50" s="88" t="s">
+        <v>214</v>
+      </c>
+      <c r="G50" s="62" t="s">
+        <v>215</v>
+      </c>
+      <c r="H50" s="62" t="s">
+        <v>216</v>
+      </c>
+      <c r="I50" s="62" t="s">
+        <v>217</v>
+      </c>
+      <c r="J50" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K50" s="89"/>
+      <c r="L50" s="89"/>
+      <c r="M50" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N50" s="110" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="38.25" customHeight="1">
+      <c r="A51" s="87"/>
+      <c r="B51" s="87"/>
+      <c r="C51" s="87"/>
+      <c r="D51" s="87"/>
+      <c r="E51" s="87"/>
+      <c r="F51" s="87"/>
+      <c r="G51" s="62" t="s">
+        <v>218</v>
+      </c>
+      <c r="H51" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I51" s="62" t="s">
+        <v>219</v>
+      </c>
+      <c r="J51" s="87"/>
+      <c r="K51" s="91"/>
+      <c r="L51" s="91"/>
+      <c r="M51" s="91"/>
+      <c r="N51" s="88"/>
+    </row>
+    <row r="52" spans="1:14" ht="38.25">
+      <c r="A52" s="87"/>
+      <c r="B52" s="87"/>
+      <c r="C52" s="87"/>
+      <c r="D52" s="87"/>
+      <c r="E52" s="87"/>
+      <c r="F52" s="87"/>
+      <c r="G52" s="62" t="s">
+        <v>220</v>
+      </c>
+      <c r="H52" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I52" s="62" t="s">
+        <v>221</v>
+      </c>
+      <c r="J52" s="87"/>
+      <c r="K52" s="91"/>
+      <c r="L52" s="91"/>
+      <c r="M52" s="91"/>
+      <c r="N52" s="88"/>
+    </row>
+    <row r="53" spans="1:14" ht="51" customHeight="1">
+      <c r="A53" s="87">
+        <v>14</v>
+      </c>
+      <c r="B53" s="88" t="s">
+        <v>222</v>
+      </c>
+      <c r="C53" s="88" t="s">
+        <v>112</v>
+      </c>
+      <c r="D53" s="88" t="s">
+        <v>223</v>
+      </c>
+      <c r="E53" s="87">
+        <v>1</v>
+      </c>
+      <c r="F53" s="88" t="s">
+        <v>224</v>
+      </c>
+      <c r="G53" s="62" t="s">
+        <v>114</v>
+      </c>
+      <c r="H53" s="62" t="s">
+        <v>225</v>
+      </c>
+      <c r="I53" s="62" t="s">
+        <v>226</v>
+      </c>
+      <c r="J53" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K53" s="89"/>
+      <c r="L53" s="89"/>
+      <c r="M53" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N53" s="110" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" ht="38.25">
+      <c r="A54" s="87"/>
+      <c r="B54" s="87"/>
+      <c r="C54" s="87"/>
+      <c r="D54" s="87"/>
+      <c r="E54" s="87"/>
+      <c r="F54" s="87"/>
+      <c r="G54" s="62" t="s">
+        <v>227</v>
+      </c>
+      <c r="H54" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I54" s="62" t="s">
+        <v>228</v>
+      </c>
+      <c r="J54" s="87"/>
+      <c r="K54" s="91"/>
+      <c r="L54" s="91"/>
+      <c r="M54" s="91"/>
+      <c r="N54" s="88"/>
+    </row>
+    <row r="55" spans="1:14" ht="89.25" customHeight="1">
+      <c r="A55" s="87">
+        <v>15</v>
+      </c>
+      <c r="B55" s="88" t="s">
+        <v>229</v>
+      </c>
+      <c r="C55" s="88" t="s">
+        <v>230</v>
+      </c>
+      <c r="D55" s="88" t="s">
+        <v>223</v>
+      </c>
+      <c r="E55" s="87">
+        <v>1</v>
+      </c>
+      <c r="F55" s="88" t="s">
+        <v>231</v>
+      </c>
+      <c r="G55" s="62" t="s">
+        <v>232</v>
+      </c>
+      <c r="H55" s="62" t="s">
+        <v>233</v>
+      </c>
+      <c r="I55" s="62" t="s">
+        <v>234</v>
+      </c>
+      <c r="J55" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="K55" s="89"/>
+      <c r="L55" s="89"/>
+      <c r="M55" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="N55" s="110" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" ht="25.5">
+      <c r="A56" s="87"/>
+      <c r="B56" s="87"/>
+      <c r="C56" s="87"/>
+      <c r="D56" s="87"/>
+      <c r="E56" s="87"/>
+      <c r="F56" s="87"/>
+      <c r="G56" s="62" t="s">
+        <v>235</v>
+      </c>
+      <c r="H56" s="62" t="s">
+        <v>236</v>
+      </c>
+      <c r="I56" s="62" t="s">
+        <v>237</v>
+      </c>
+      <c r="J56" s="87"/>
+      <c r="K56" s="91"/>
+      <c r="L56" s="91"/>
+      <c r="M56" s="91"/>
+      <c r="N56" s="88"/>
+    </row>
+    <row r="57" spans="1:14" ht="38.25">
+      <c r="A57" s="87"/>
+      <c r="B57" s="87"/>
+      <c r="C57" s="87"/>
+      <c r="D57" s="87"/>
+      <c r="E57" s="87"/>
+      <c r="F57" s="87"/>
+      <c r="G57" s="62" t="s">
+        <v>238</v>
+      </c>
+      <c r="H57" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="I57" s="62" t="s">
+        <v>239</v>
+      </c>
+      <c r="J57" s="87"/>
+      <c r="K57" s="91"/>
+      <c r="L57" s="91"/>
+      <c r="M57" s="91"/>
+      <c r="N57" s="88"/>
+    </row>
+    <row r="58" spans="1:14">
       <c r="A58" s="21"/>
       <c r="B58" s="21"/>
       <c r="C58" s="21"/>
@@ -4748,7 +5522,7 @@
       <c r="I58" s="21"/>
       <c r="J58" s="21"/>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:14">
       <c r="A59" s="21"/>
       <c r="B59" s="21"/>
       <c r="C59" s="21"/>
@@ -4760,7 +5534,7 @@
       <c r="I59" s="21"/>
       <c r="J59" s="21"/>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:14">
       <c r="A60" s="21"/>
       <c r="B60" s="21"/>
       <c r="C60" s="21"/>
@@ -4772,7 +5546,7 @@
       <c r="I60" s="21"/>
       <c r="J60" s="21"/>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:14">
       <c r="A61" s="21"/>
       <c r="B61" s="21"/>
       <c r="C61" s="21"/>
@@ -4784,7 +5558,7 @@
       <c r="I61" s="21"/>
       <c r="J61" s="21"/>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:14">
       <c r="A62" s="21"/>
       <c r="B62" s="21"/>
       <c r="C62" s="21"/>
@@ -4796,7 +5570,7 @@
       <c r="I62" s="21"/>
       <c r="J62" s="21"/>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:14">
       <c r="A63" s="21"/>
       <c r="B63" s="21"/>
       <c r="C63" s="21"/>
@@ -4808,7 +5582,7 @@
       <c r="I63" s="21"/>
       <c r="J63" s="21"/>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:14">
       <c r="A64" s="21"/>
       <c r="B64" s="21"/>
       <c r="C64" s="21"/>
@@ -5913,18 +6687,174 @@
     </row>
   </sheetData>
   <autoFilter ref="A12:N13" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <mergeCells count="95">
-    <mergeCell ref="N29:N30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="K29:K30"/>
-    <mergeCell ref="L29:L30"/>
-    <mergeCell ref="M29:M30"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E29:E30"/>
+  <mergeCells count="194">
+    <mergeCell ref="L55:L57"/>
+    <mergeCell ref="M55:M57"/>
+    <mergeCell ref="A55:A57"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="D55:D57"/>
+    <mergeCell ref="K55:K57"/>
+    <mergeCell ref="D50:D52"/>
+    <mergeCell ref="K50:K52"/>
+    <mergeCell ref="L50:L52"/>
+    <mergeCell ref="M50:M52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="K53:K54"/>
+    <mergeCell ref="L53:L54"/>
+    <mergeCell ref="M53:M54"/>
+    <mergeCell ref="K43:K45"/>
+    <mergeCell ref="L43:L45"/>
+    <mergeCell ref="M43:M45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="K46:K49"/>
+    <mergeCell ref="L46:L49"/>
+    <mergeCell ref="M46:M49"/>
+    <mergeCell ref="K36:K38"/>
+    <mergeCell ref="L36:L38"/>
+    <mergeCell ref="M36:M38"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="C39:C42"/>
+    <mergeCell ref="D39:D42"/>
+    <mergeCell ref="K39:K42"/>
+    <mergeCell ref="L39:L42"/>
+    <mergeCell ref="M39:M42"/>
+    <mergeCell ref="K31:K33"/>
+    <mergeCell ref="L31:L33"/>
+    <mergeCell ref="M31:M33"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="K34:K35"/>
+    <mergeCell ref="L34:L35"/>
+    <mergeCell ref="M34:M35"/>
+    <mergeCell ref="J55:J57"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="D36:D38"/>
+    <mergeCell ref="A43:A45"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="A50:A52"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="E55:E57"/>
+    <mergeCell ref="F55:F57"/>
+    <mergeCell ref="J50:J52"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="J53:J54"/>
+    <mergeCell ref="E50:E52"/>
+    <mergeCell ref="F50:F52"/>
+    <mergeCell ref="J43:J45"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="J46:J49"/>
+    <mergeCell ref="E43:E45"/>
+    <mergeCell ref="F43:F45"/>
+    <mergeCell ref="J36:J38"/>
+    <mergeCell ref="E39:E42"/>
+    <mergeCell ref="F39:F42"/>
+    <mergeCell ref="J39:J42"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="F31:F33"/>
+    <mergeCell ref="J31:J33"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="J34:J35"/>
+    <mergeCell ref="E36:E38"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="N55:N57"/>
+    <mergeCell ref="N53:N54"/>
+    <mergeCell ref="N50:N52"/>
+    <mergeCell ref="N46:N49"/>
+    <mergeCell ref="N43:N45"/>
+    <mergeCell ref="N39:N42"/>
+    <mergeCell ref="N36:N38"/>
+    <mergeCell ref="N34:N35"/>
+    <mergeCell ref="N31:N33"/>
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:N11"/>
+    <mergeCell ref="J12:N12"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="D8:I8"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="N16:N17"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M18:M20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="N18:N20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="J21:J23"/>
+    <mergeCell ref="K21:K23"/>
+    <mergeCell ref="L21:L23"/>
+    <mergeCell ref="M21:M23"/>
+    <mergeCell ref="N21:N23"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="J18:J20"/>
+    <mergeCell ref="K18:K20"/>
+    <mergeCell ref="L18:L20"/>
+    <mergeCell ref="M24:M26"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="E24:E26"/>
     <mergeCell ref="N24:N26"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
@@ -5941,74 +6871,17 @@
     <mergeCell ref="J24:J26"/>
     <mergeCell ref="K24:K26"/>
     <mergeCell ref="L24:L26"/>
-    <mergeCell ref="M24:M26"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="N18:N20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="C21:C23"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="F21:F23"/>
-    <mergeCell ref="J21:J23"/>
-    <mergeCell ref="K21:K23"/>
-    <mergeCell ref="L21:L23"/>
-    <mergeCell ref="M21:M23"/>
-    <mergeCell ref="N21:N23"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="J18:J20"/>
-    <mergeCell ref="K18:K20"/>
-    <mergeCell ref="L18:L20"/>
-    <mergeCell ref="M18:M20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="M16:M17"/>
-    <mergeCell ref="N16:N17"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="D9:I9"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:N11"/>
-    <mergeCell ref="J12:N12"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="D6:I6"/>
-    <mergeCell ref="D7:I7"/>
-    <mergeCell ref="D8:I8"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="N29:N30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="K29:K30"/>
+    <mergeCell ref="L29:L30"/>
+    <mergeCell ref="M29:M30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6037,7 +6910,7 @@
         <v>67</v>
       </c>
       <c r="C4" s="22">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="2:4">
@@ -6061,7 +6934,7 @@
         <v>70</v>
       </c>
       <c r="C11" s="22">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:4">
@@ -6101,6 +6974,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AF28BDBD65D93F4BA99B6439AFEA320E" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="11d45d99e0339591c68aad091688ac92">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9b0ef35d-78e7-41bf-847f-3c0497ad5352" xmlns:ns3="3c969135-7855-44e0-a9fe-01d799f07605" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e603a3f7bf67670d682b80385fe4b00" ns2:_="" ns3:_="">
     <xsd:import namespace="9b0ef35d-78e7-41bf-847f-3c0497ad5352"/>
@@ -6301,22 +7189,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFD7E773-5319-49CF-80DA-12E24FC51CD2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5F7A0BD-DCD4-473A-A4BF-DC65A831158E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0FD9AFA-8FB8-4A5A-8D3C-E657A5B7F741}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6333,21 +7223,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5F7A0BD-DCD4-473A-A4BF-DC65A831158E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFD7E773-5319-49CF-80DA-12E24FC51CD2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>